<commit_message>
WS_Mdl re-format #14: NBr52 running (debugged)
</commit_message>
<xml_diff>
--- a/Mng/Acronyms.xlsx
+++ b/Mng/Acronyms.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Mng\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB9D7C76-1884-481B-92AE-FB6B6187BD0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8DFF767-AA5C-4033-B498-429BCF972505}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-165" yWindow="-165" windowWidth="29130" windowHeight="15810" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Acronyms" sheetId="1" r:id="rId1"/>
@@ -307,7 +307,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1869" uniqueCount="850">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1054" uniqueCount="852">
   <si>
     <t>GW</t>
   </si>
@@ -2858,6 +2858,13 @@
   </si>
   <si>
     <t>Separator</t>
+  </si>
+  <si>
+    <t>Model</t>
+  </si>
+  <si>
+    <t>Different context to other M.
+Needed for WS_Mdl python lib, where MdlN is used as an arg, Mdl_N is a class, so M is the instance of this class based on the arg. Using M for this makes it very easy to reference.</t>
   </si>
 </sst>
 </file>
@@ -2955,7 +2962,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2993,6 +3000,9 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -9818,10 +9828,18 @@
         <v/>
       </c>
     </row>
-    <row r="418" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B418" s="5"/>
+    <row r="418" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+      <c r="A418" s="5" t="s">
+        <v>280</v>
+      </c>
+      <c r="B418" s="5" t="s">
+        <v>850</v>
+      </c>
       <c r="C418" s="5" t="s">
-        <v>156</v>
+        <v>423</v>
+      </c>
+      <c r="D418" s="17" t="s">
+        <v>851</v>
       </c>
       <c r="E418" t="str">
         <f t="shared" si="12"/>

</xml_diff>

<commit_message>
NBr100-102 finished + PoP started
</commit_message>
<xml_diff>
--- a/Mng/Acronyms.xlsx
+++ b/Mng/Acronyms.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Mng\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1D4AB3A-6499-4EF5-A742-D418C8015072}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C912A69D-99BE-47FE-9E96-271DF7B7A24D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -307,7 +307,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1874" uniqueCount="856">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4294947668" uniqueCount="856">
   <si>
     <t>GW</t>
   </si>
@@ -1573,9 +1573,6 @@
     <t>Statistics</t>
   </si>
   <si>
-    <t>l</t>
-  </si>
-  <si>
     <t>list</t>
   </si>
   <si>
@@ -2877,6 +2874,9 @@
   </si>
   <si>
     <t>Decline</t>
+  </si>
+  <si>
+    <t>l_</t>
   </si>
 </sst>
 </file>
@@ -3448,7 +3448,7 @@
         <v>155</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>81</v>
@@ -3473,15 +3473,15 @@
       </c>
       <c r="F2" s="4">
         <f>SUM(E2:E994)</f>
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>292</v>
@@ -3493,13 +3493,13 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
+        <v>755</v>
+      </c>
+      <c r="B4" s="5" t="s">
         <v>756</v>
       </c>
-      <c r="B4" s="5" t="s">
-        <v>757</v>
-      </c>
       <c r="C4" s="5" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E4" t="str">
         <f t="shared" si="0"/>
@@ -3508,13 +3508,13 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
+        <v>639</v>
+      </c>
+      <c r="B5" s="5" t="s">
         <v>640</v>
       </c>
-      <c r="B5" s="5" t="s">
-        <v>641</v>
-      </c>
       <c r="C5" s="5" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E5" t="str">
         <f t="shared" si="0"/>
@@ -3711,7 +3711,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="B18" s="5" t="s">
         <v>58</v>
@@ -3727,10 +3727,10 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
+        <v>450</v>
+      </c>
+      <c r="B19" s="5" t="s">
         <v>451</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>452</v>
       </c>
       <c r="C19" s="5" t="s">
         <v>300</v>
@@ -3757,16 +3757,16 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="C21" s="5" t="s">
         <v>300</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="E21" t="str">
         <f t="shared" si="0"/>
@@ -3791,16 +3791,16 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
+        <v>786</v>
+      </c>
+      <c r="B23" s="5" t="s">
         <v>787</v>
-      </c>
-      <c r="B23" s="5" t="s">
-        <v>788</v>
       </c>
       <c r="C23" s="5" t="s">
         <v>300</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="E23" t="str">
         <f t="shared" si="0"/>
@@ -3824,7 +3824,7 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="B25" s="5" t="s">
         <v>51</v>
@@ -3843,7 +3843,7 @@
         <v>356</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
       <c r="C26" s="5" t="s">
         <v>290</v>
@@ -3855,10 +3855,10 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
+        <v>841</v>
+      </c>
+      <c r="B27" s="5" t="s">
         <v>842</v>
-      </c>
-      <c r="B27" s="5" t="s">
-        <v>843</v>
       </c>
       <c r="C27" s="5" t="s">
         <v>292</v>
@@ -3886,10 +3886,10 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
+        <v>607</v>
+      </c>
+      <c r="B29" s="5" t="s">
         <v>608</v>
-      </c>
-      <c r="B29" s="5" t="s">
-        <v>609</v>
       </c>
       <c r="C29" s="5" t="s">
         <v>292</v>
@@ -3901,10 +3901,10 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
+        <v>793</v>
+      </c>
+      <c r="B30" s="5" t="s">
         <v>794</v>
-      </c>
-      <c r="B30" s="5" t="s">
-        <v>795</v>
       </c>
       <c r="C30" s="5" t="s">
         <v>292</v>
@@ -3931,10 +3931,10 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
+        <v>751</v>
+      </c>
+      <c r="B32" s="5" t="s">
         <v>752</v>
-      </c>
-      <c r="B32" s="5" t="s">
-        <v>753</v>
       </c>
       <c r="C32" s="5" t="s">
         <v>292</v>
@@ -3946,10 +3946,10 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
+        <v>749</v>
+      </c>
+      <c r="B33" s="5" t="s">
         <v>750</v>
-      </c>
-      <c r="B33" s="5" t="s">
-        <v>751</v>
       </c>
       <c r="C33" s="5" t="s">
         <v>300</v>
@@ -3977,13 +3977,13 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
+        <v>769</v>
+      </c>
+      <c r="B35" s="5" t="s">
         <v>770</v>
       </c>
-      <c r="B35" s="5" t="s">
-        <v>771</v>
-      </c>
       <c r="C35" s="5" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E35" t="str">
         <f t="shared" si="1"/>
@@ -3992,10 +3992,10 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="s">
+        <v>626</v>
+      </c>
+      <c r="B36" s="5" t="s">
         <v>627</v>
-      </c>
-      <c r="B36" s="5" t="s">
-        <v>628</v>
       </c>
       <c r="C36" s="5" t="s">
         <v>300</v>
@@ -4007,13 +4007,13 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="11" t="s">
+        <v>545</v>
+      </c>
+      <c r="B37" s="11" t="s">
         <v>546</v>
       </c>
-      <c r="B37" s="11" t="s">
-        <v>547</v>
-      </c>
       <c r="C37" s="5" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="E37" t="str">
         <f t="shared" si="1"/>
@@ -4068,10 +4068,10 @@
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="5" t="s">
+        <v>497</v>
+      </c>
+      <c r="B41" s="5" t="s">
         <v>498</v>
-      </c>
-      <c r="B41" s="5" t="s">
-        <v>499</v>
       </c>
       <c r="C41" s="5" t="s">
         <v>292</v>
@@ -4083,10 +4083,10 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
+        <v>702</v>
+      </c>
+      <c r="B42" s="5" t="s">
         <v>703</v>
-      </c>
-      <c r="B42" s="5" t="s">
-        <v>704</v>
       </c>
       <c r="C42" s="5" t="s">
         <v>300</v>
@@ -4098,10 +4098,10 @@
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
+        <v>672</v>
+      </c>
+      <c r="B43" s="5" t="s">
         <v>673</v>
-      </c>
-      <c r="B43" s="5" t="s">
-        <v>674</v>
       </c>
       <c r="C43" s="5" t="s">
         <v>292</v>
@@ -4113,10 +4113,10 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
+        <v>700</v>
+      </c>
+      <c r="B44" s="5" t="s">
         <v>701</v>
-      </c>
-      <c r="B44" s="5" t="s">
-        <v>702</v>
       </c>
       <c r="C44" s="5" t="s">
         <v>300</v>
@@ -4128,10 +4128,10 @@
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="11" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="B45" s="12" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="C45" s="5" t="s">
         <v>292</v>
@@ -4143,10 +4143,10 @@
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
       <c r="C46" s="5" t="s">
         <v>300</v>
@@ -4158,10 +4158,10 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="s">
+        <v>816</v>
+      </c>
+      <c r="B47" s="5" t="s">
         <v>817</v>
-      </c>
-      <c r="B47" s="5" t="s">
-        <v>818</v>
       </c>
       <c r="C47" s="5" t="s">
         <v>300</v>
@@ -4173,10 +4173,10 @@
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="5" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="C48" s="5" t="s">
         <v>300</v>
@@ -4188,10 +4188,10 @@
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="5" t="s">
+        <v>742</v>
+      </c>
+      <c r="B49" s="5" t="s">
         <v>743</v>
-      </c>
-      <c r="B49" s="5" t="s">
-        <v>744</v>
       </c>
       <c r="C49" s="5" t="s">
         <v>300</v>
@@ -4203,10 +4203,10 @@
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="5" t="s">
+        <v>461</v>
+      </c>
+      <c r="B50" s="5" t="s">
         <v>462</v>
-      </c>
-      <c r="B50" s="5" t="s">
-        <v>463</v>
       </c>
       <c r="C50" s="5" t="s">
         <v>292</v>
@@ -4218,13 +4218,13 @@
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="5" t="s">
+        <v>803</v>
+      </c>
+      <c r="B51" s="5" t="s">
         <v>804</v>
       </c>
-      <c r="B51" s="5" t="s">
-        <v>805</v>
-      </c>
       <c r="C51" s="5" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E51" t="str">
         <f t="shared" si="1"/>
@@ -4233,10 +4233,10 @@
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="5" t="s">
+        <v>687</v>
+      </c>
+      <c r="B52" s="5" t="s">
         <v>688</v>
-      </c>
-      <c r="B52" s="5" t="s">
-        <v>689</v>
       </c>
       <c r="C52" s="5" t="s">
         <v>292</v>
@@ -4267,10 +4267,10 @@
         <v>275</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E54">
         <f t="shared" si="1"/>
@@ -4282,7 +4282,7 @@
         <v>275</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="C55" s="5" t="s">
         <v>293</v>
@@ -4294,10 +4294,10 @@
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="5" t="s">
+        <v>818</v>
+      </c>
+      <c r="B56" s="5" t="s">
         <v>819</v>
-      </c>
-      <c r="B56" s="5" t="s">
-        <v>820</v>
       </c>
       <c r="C56" s="5" t="s">
         <v>300</v>
@@ -4345,10 +4345,10 @@
         <v>260</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E59">
         <f t="shared" si="1"/>
@@ -4357,10 +4357,10 @@
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="11" t="s">
+        <v>595</v>
+      </c>
+      <c r="B60" s="12" t="s">
         <v>596</v>
-      </c>
-      <c r="B60" s="12" t="s">
-        <v>597</v>
       </c>
       <c r="C60" s="5" t="s">
         <v>292</v>
@@ -4372,10 +4372,10 @@
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="5" t="s">
+        <v>853</v>
+      </c>
+      <c r="B61" s="5" t="s">
         <v>854</v>
-      </c>
-      <c r="B61" s="5" t="s">
-        <v>855</v>
       </c>
       <c r="E61" t="str">
         <f t="shared" si="1"/>
@@ -4384,10 +4384,10 @@
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" s="5" t="s">
+        <v>635</v>
+      </c>
+      <c r="B62" s="5" t="s">
         <v>636</v>
-      </c>
-      <c r="B62" s="5" t="s">
-        <v>637</v>
       </c>
       <c r="C62" s="5" t="s">
         <v>300</v>
@@ -4414,13 +4414,13 @@
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="5" t="s">
+        <v>430</v>
+      </c>
+      <c r="B64" s="5" t="s">
         <v>431</v>
       </c>
-      <c r="B64" s="5" t="s">
-        <v>432</v>
-      </c>
       <c r="C64" s="5" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E64" t="str">
         <f t="shared" si="1"/>
@@ -4429,10 +4429,10 @@
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="5" t="s">
+        <v>452</v>
+      </c>
+      <c r="B65" s="5" t="s">
         <v>453</v>
-      </c>
-      <c r="B65" s="5" t="s">
-        <v>454</v>
       </c>
       <c r="C65" s="5" t="s">
         <v>182</v>
@@ -4460,10 +4460,10 @@
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="5" t="s">
+        <v>661</v>
+      </c>
+      <c r="B67" s="5" t="s">
         <v>662</v>
-      </c>
-      <c r="B67" s="5" t="s">
-        <v>663</v>
       </c>
       <c r="C67" s="5" t="s">
         <v>300</v>
@@ -4490,13 +4490,13 @@
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="5" t="s">
+        <v>441</v>
+      </c>
+      <c r="B69" s="5" t="s">
         <v>442</v>
       </c>
-      <c r="B69" s="5" t="s">
-        <v>443</v>
-      </c>
       <c r="C69" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="E69" t="str">
         <f t="shared" si="2"/>
@@ -4520,13 +4520,13 @@
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="11" t="s">
+        <v>565</v>
+      </c>
+      <c r="B71" s="11" t="s">
         <v>566</v>
       </c>
-      <c r="B71" s="11" t="s">
-        <v>567</v>
-      </c>
       <c r="C71" s="5" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="E71">
         <f t="shared" si="2"/>
@@ -4535,10 +4535,10 @@
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="5" t="s">
+        <v>795</v>
+      </c>
+      <c r="B72" s="5" t="s">
         <v>796</v>
-      </c>
-      <c r="B72" s="5" t="s">
-        <v>797</v>
       </c>
       <c r="C72" s="5" t="s">
         <v>300</v>
@@ -4550,13 +4550,13 @@
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="11" t="s">
+        <v>569</v>
+      </c>
+      <c r="B73" s="11" t="s">
         <v>570</v>
       </c>
-      <c r="B73" s="11" t="s">
-        <v>571</v>
-      </c>
       <c r="C73" s="5" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="E73" t="str">
         <f t="shared" si="2"/>
@@ -4565,13 +4565,13 @@
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="11" t="s">
+        <v>567</v>
+      </c>
+      <c r="B74" s="11" t="s">
         <v>568</v>
       </c>
-      <c r="B74" s="11" t="s">
-        <v>569</v>
-      </c>
       <c r="C74" s="5" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="E74" t="str">
         <f t="shared" si="2"/>
@@ -4580,10 +4580,10 @@
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" s="5" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="B75" s="5" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="C75" s="5" t="s">
         <v>300</v>
@@ -4595,10 +4595,10 @@
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="5" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="B76" s="5" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="C76" s="5" t="s">
         <v>292</v>
@@ -4655,13 +4655,13 @@
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="11" t="s">
+        <v>549</v>
+      </c>
+      <c r="B80" s="11" t="s">
         <v>550</v>
       </c>
-      <c r="B80" s="11" t="s">
-        <v>551</v>
-      </c>
       <c r="C80" s="5" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="E80">
         <f t="shared" si="2"/>
@@ -4685,10 +4685,10 @@
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" s="5" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="B82" s="5" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="C82" s="5" t="s">
         <v>292</v>
@@ -4700,10 +4700,10 @@
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" s="5" t="s">
+        <v>744</v>
+      </c>
+      <c r="B83" s="5" t="s">
         <v>745</v>
-      </c>
-      <c r="B83" s="5" t="s">
-        <v>746</v>
       </c>
       <c r="C83" s="5" t="s">
         <v>292</v>
@@ -4715,10 +4715,10 @@
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="5" t="s">
+        <v>503</v>
+      </c>
+      <c r="B84" s="5" t="s">
         <v>504</v>
-      </c>
-      <c r="B84" s="5" t="s">
-        <v>505</v>
       </c>
       <c r="C84" s="5" t="s">
         <v>300</v>
@@ -4872,10 +4872,10 @@
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" s="5" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="B94" s="5" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="C94" s="5" t="s">
         <v>292</v>
@@ -4917,10 +4917,10 @@
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" s="5" t="s">
+        <v>713</v>
+      </c>
+      <c r="B97" s="5" t="s">
         <v>714</v>
-      </c>
-      <c r="B97" s="5" t="s">
-        <v>715</v>
       </c>
       <c r="C97" s="5" t="s">
         <v>300</v>
@@ -4948,10 +4948,10 @@
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" s="5" t="s">
+        <v>620</v>
+      </c>
+      <c r="B99" s="5" t="s">
         <v>621</v>
-      </c>
-      <c r="B99" s="5" t="s">
-        <v>622</v>
       </c>
       <c r="C99" s="5" t="s">
         <v>300</v>
@@ -4993,10 +4993,10 @@
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" s="5" t="s">
+        <v>491</v>
+      </c>
+      <c r="B102" s="5" t="s">
         <v>492</v>
-      </c>
-      <c r="B102" s="5" t="s">
-        <v>493</v>
       </c>
       <c r="C102" s="5" t="s">
         <v>300</v>
@@ -5008,13 +5008,13 @@
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" s="11" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="B103" s="11" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="C103" s="5" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="E103">
         <f t="shared" si="3"/>
@@ -5023,10 +5023,10 @@
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" s="5" t="s">
+        <v>830</v>
+      </c>
+      <c r="B104" s="5" t="s">
         <v>831</v>
-      </c>
-      <c r="B104" s="5" t="s">
-        <v>832</v>
       </c>
       <c r="C104" s="5" t="s">
         <v>300</v>
@@ -5038,10 +5038,10 @@
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A105" s="5" t="s">
+        <v>637</v>
+      </c>
+      <c r="B105" s="5" t="s">
         <v>638</v>
-      </c>
-      <c r="B105" s="5" t="s">
-        <v>639</v>
       </c>
       <c r="C105" s="5" t="s">
         <v>292</v>
@@ -5099,10 +5099,10 @@
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A109" s="5" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="B109" s="5" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="C109" s="5" t="s">
         <v>292</v>
@@ -5114,10 +5114,10 @@
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A110" s="5" t="s">
+        <v>477</v>
+      </c>
+      <c r="B110" s="5" t="s">
         <v>478</v>
-      </c>
-      <c r="B110" s="5" t="s">
-        <v>479</v>
       </c>
       <c r="C110" s="5" t="s">
         <v>292</v>
@@ -5129,10 +5129,10 @@
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A111" s="5" t="s">
+        <v>537</v>
+      </c>
+      <c r="B111" s="5" t="s">
         <v>538</v>
-      </c>
-      <c r="B111" s="5" t="s">
-        <v>539</v>
       </c>
       <c r="C111" s="5" t="s">
         <v>292</v>
@@ -5159,10 +5159,10 @@
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113" s="5" t="s">
+        <v>685</v>
+      </c>
+      <c r="B113" s="5" t="s">
         <v>686</v>
-      </c>
-      <c r="B113" s="5" t="s">
-        <v>687</v>
       </c>
       <c r="C113" s="5" t="s">
         <v>300</v>
@@ -5174,10 +5174,10 @@
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A114" s="5" t="s">
+        <v>469</v>
+      </c>
+      <c r="B114" s="5" t="s">
         <v>470</v>
-      </c>
-      <c r="B114" s="5" t="s">
-        <v>471</v>
       </c>
       <c r="C114" s="5" t="s">
         <v>290</v>
@@ -5189,10 +5189,10 @@
     </row>
     <row r="115" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A115" s="5" t="s">
+        <v>706</v>
+      </c>
+      <c r="B115" s="5" t="s">
         <v>707</v>
-      </c>
-      <c r="B115" s="5" t="s">
-        <v>708</v>
       </c>
       <c r="C115" s="5" t="s">
         <v>300</v>
@@ -5204,10 +5204,10 @@
     </row>
     <row r="116" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A116" s="5" t="s">
+        <v>717</v>
+      </c>
+      <c r="B116" s="5" t="s">
         <v>718</v>
-      </c>
-      <c r="B116" s="5" t="s">
-        <v>719</v>
       </c>
       <c r="C116" s="5" t="s">
         <v>300</v>
@@ -5219,10 +5219,10 @@
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117" s="5" t="s">
+        <v>433</v>
+      </c>
+      <c r="B117" s="5" t="s">
         <v>434</v>
-      </c>
-      <c r="B117" s="5" t="s">
-        <v>435</v>
       </c>
       <c r="C117" s="5" t="s">
         <v>292</v>
@@ -5234,13 +5234,13 @@
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="B118" s="5" t="s">
         <v>439</v>
       </c>
-      <c r="B118" s="5" t="s">
+      <c r="C118" s="5" t="s">
         <v>440</v>
-      </c>
-      <c r="C118" s="5" t="s">
-        <v>441</v>
       </c>
       <c r="E118" t="str">
         <f t="shared" si="3"/>
@@ -5312,10 +5312,10 @@
     </row>
     <row r="123" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A123" s="5" t="s">
+        <v>776</v>
+      </c>
+      <c r="B123" s="5" t="s">
         <v>777</v>
-      </c>
-      <c r="B123" s="5" t="s">
-        <v>778</v>
       </c>
       <c r="C123" s="5" t="s">
         <v>292</v>
@@ -5327,7 +5327,7 @@
     </row>
     <row r="124" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A124" s="5" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="B124" s="5" t="s">
         <v>301</v>
@@ -5342,10 +5342,10 @@
     </row>
     <row r="125" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A125" s="5" t="s">
+        <v>467</v>
+      </c>
+      <c r="B125" s="5" t="s">
         <v>468</v>
-      </c>
-      <c r="B125" s="5" t="s">
-        <v>469</v>
       </c>
       <c r="C125" s="5" t="s">
         <v>292</v>
@@ -5357,13 +5357,13 @@
     </row>
     <row r="126" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A126" s="11" t="s">
+        <v>552</v>
+      </c>
+      <c r="B126" s="11" t="s">
         <v>553</v>
       </c>
-      <c r="B126" s="11" t="s">
-        <v>554</v>
-      </c>
       <c r="C126" s="5" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="E126" t="str">
         <f t="shared" si="3"/>
@@ -5437,13 +5437,13 @@
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A131" s="11" t="s">
+        <v>582</v>
+      </c>
+      <c r="B131" s="11" t="s">
         <v>583</v>
       </c>
-      <c r="B131" s="11" t="s">
-        <v>584</v>
-      </c>
       <c r="C131" s="5" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="E131" t="str">
         <f t="shared" si="4"/>
@@ -5467,10 +5467,10 @@
     </row>
     <row r="133" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A133" s="5" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="B133" s="5" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="C133" s="5" t="s">
         <v>300</v>
@@ -5482,10 +5482,10 @@
     </row>
     <row r="134" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A134" s="5" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
       <c r="B134" s="5" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="C134" s="5" t="s">
         <v>292</v>
@@ -5604,10 +5604,10 @@
     </row>
     <row r="142" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A142" s="5" t="s">
+        <v>481</v>
+      </c>
+      <c r="B142" s="5" t="s">
         <v>482</v>
-      </c>
-      <c r="B142" s="5" t="s">
-        <v>483</v>
       </c>
       <c r="C142" s="5" t="s">
         <v>292</v>
@@ -5726,10 +5726,10 @@
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A150" s="5" t="s">
+        <v>459</v>
+      </c>
+      <c r="B150" s="5" t="s">
         <v>460</v>
-      </c>
-      <c r="B150" s="5" t="s">
-        <v>461</v>
       </c>
       <c r="C150" s="5" t="s">
         <v>292</v>
@@ -5759,7 +5759,7 @@
         <v>311</v>
       </c>
       <c r="B152" s="5" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="C152" s="5" t="s">
         <v>292</v>
@@ -5801,10 +5801,10 @@
     </row>
     <row r="155" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A155" s="5" t="s">
+        <v>610</v>
+      </c>
+      <c r="B155" s="5" t="s">
         <v>611</v>
-      </c>
-      <c r="B155" s="5" t="s">
-        <v>612</v>
       </c>
       <c r="C155" s="5" t="s">
         <v>292</v>
@@ -5816,10 +5816,10 @@
     </row>
     <row r="156" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A156" s="5" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="B156" s="5" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="C156" s="5" t="s">
         <v>300</v>
@@ -5846,10 +5846,10 @@
     </row>
     <row r="158" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A158" s="5" t="s">
+        <v>837</v>
+      </c>
+      <c r="B158" s="5" t="s">
         <v>838</v>
-      </c>
-      <c r="B158" s="5" t="s">
-        <v>839</v>
       </c>
       <c r="C158" s="5" t="s">
         <v>292</v>
@@ -5861,13 +5861,13 @@
     </row>
     <row r="159" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A159" s="11" t="s">
+        <v>574</v>
+      </c>
+      <c r="B159" s="11" t="s">
         <v>575</v>
       </c>
-      <c r="B159" s="11" t="s">
-        <v>576</v>
-      </c>
       <c r="C159" s="5" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="E159" t="str">
         <f t="shared" si="4"/>
@@ -5876,10 +5876,10 @@
     </row>
     <row r="160" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A160" s="5" t="s">
+        <v>674</v>
+      </c>
+      <c r="B160" s="5" t="s">
         <v>675</v>
-      </c>
-      <c r="B160" s="5" t="s">
-        <v>676</v>
       </c>
       <c r="C160" s="5" t="s">
         <v>300</v>
@@ -5921,13 +5921,13 @@
     </row>
     <row r="163" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A163" s="11" t="s">
+        <v>584</v>
+      </c>
+      <c r="B163" s="11" t="s">
         <v>585</v>
       </c>
-      <c r="B163" s="11" t="s">
-        <v>586</v>
-      </c>
       <c r="C163" s="5" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="E163" t="str">
         <f t="shared" si="5"/>
@@ -5936,16 +5936,16 @@
     </row>
     <row r="164" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A164" s="5" t="s">
+        <v>523</v>
+      </c>
+      <c r="B164" s="5" t="s">
         <v>524</v>
       </c>
-      <c r="B164" s="5" t="s">
-        <v>525</v>
-      </c>
       <c r="C164" s="5" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="D164" s="5" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="E164" t="str">
         <f t="shared" si="5"/>
@@ -5969,10 +5969,10 @@
     </row>
     <row r="166" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A166" s="5" t="s">
+        <v>851</v>
+      </c>
+      <c r="B166" s="5" t="s">
         <v>852</v>
-      </c>
-      <c r="B166" s="5" t="s">
-        <v>853</v>
       </c>
       <c r="E166" t="str">
         <f t="shared" si="5"/>
@@ -5996,10 +5996,10 @@
     </row>
     <row r="168" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A168" s="5" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
       <c r="B168" s="5" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="C168" s="5" t="s">
         <v>292</v>
@@ -6011,10 +6011,10 @@
     </row>
     <row r="169" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A169" s="5" t="s">
+        <v>681</v>
+      </c>
+      <c r="B169" s="5" t="s">
         <v>682</v>
-      </c>
-      <c r="B169" s="5" t="s">
-        <v>683</v>
       </c>
       <c r="C169" s="5" t="s">
         <v>300</v>
@@ -6026,13 +6026,13 @@
     </row>
     <row r="170" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A170" s="5" t="s">
+        <v>428</v>
+      </c>
+      <c r="B170" s="5" t="s">
         <v>429</v>
       </c>
-      <c r="B170" s="5" t="s">
-        <v>430</v>
-      </c>
       <c r="C170" s="5" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E170" t="str">
         <f t="shared" si="5"/>
@@ -6041,10 +6041,10 @@
     </row>
     <row r="171" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A171" s="5" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="B171" s="5" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="C171" s="5" t="s">
         <v>300</v>
@@ -6056,10 +6056,10 @@
     </row>
     <row r="172" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A172" s="5" t="s">
+        <v>495</v>
+      </c>
+      <c r="B172" s="5" t="s">
         <v>496</v>
-      </c>
-      <c r="B172" s="5" t="s">
-        <v>497</v>
       </c>
       <c r="C172" s="5" t="s">
         <v>300</v>
@@ -6086,10 +6086,10 @@
     </row>
     <row r="174" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A174" s="5" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="B174" s="5" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="C174" s="5" t="s">
         <v>292</v>
@@ -6097,10 +6097,10 @@
     </row>
     <row r="175" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A175" s="5" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="B175" s="5" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="C175" s="5" t="s">
         <v>300</v>
@@ -6112,10 +6112,10 @@
     </row>
     <row r="176" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A176" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="B176" s="5" t="s">
         <v>634</v>
-      </c>
-      <c r="B176" s="5" t="s">
-        <v>635</v>
       </c>
       <c r="C176" s="5" t="s">
         <v>292</v>
@@ -6188,7 +6188,7 @@
         <v>296</v>
       </c>
       <c r="D180" s="5" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
       <c r="E180" t="str">
         <f t="shared" si="6"/>
@@ -6197,17 +6197,17 @@
     </row>
     <row r="181" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A181" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="B181" s="5" t="s">
         <v>421</v>
       </c>
-      <c r="B181" s="5" t="s">
+      <c r="C181" s="5" t="s">
         <v>422</v>
       </c>
-      <c r="C181" s="5" t="s">
-        <v>423</v>
-      </c>
-      <c r="E181">
+      <c r="E181" t="str">
         <f t="shared" si="6"/>
-        <v>1</v>
+        <v/>
       </c>
     </row>
     <row r="182" spans="1:5" x14ac:dyDescent="0.25">
@@ -6215,25 +6215,25 @@
         <v>294</v>
       </c>
       <c r="B182" s="5" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="C182" s="5" t="s">
         <v>292</v>
       </c>
-      <c r="E182">
+      <c r="E182" t="str">
         <f t="shared" si="6"/>
-        <v>1</v>
+        <v/>
       </c>
     </row>
     <row r="183" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A183" s="11" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="B183" s="11" t="s">
         <v>173</v>
       </c>
       <c r="C183" s="5" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="E183" t="str">
         <f t="shared" si="6"/>
@@ -6242,10 +6242,10 @@
     </row>
     <row r="184" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A184" s="5" t="s">
+        <v>521</v>
+      </c>
+      <c r="B184" s="5" t="s">
         <v>522</v>
-      </c>
-      <c r="B184" s="5" t="s">
-        <v>523</v>
       </c>
       <c r="C184" s="5" t="s">
         <v>292</v>
@@ -6257,10 +6257,10 @@
     </row>
     <row r="185" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A185" s="5" t="s">
+        <v>479</v>
+      </c>
+      <c r="B185" s="5" t="s">
         <v>480</v>
-      </c>
-      <c r="B185" s="5" t="s">
-        <v>481</v>
       </c>
       <c r="C185" s="5" t="s">
         <v>300</v>
@@ -6287,13 +6287,13 @@
     </row>
     <row r="187" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A187" s="11" t="s">
+        <v>588</v>
+      </c>
+      <c r="B187" s="11" t="s">
         <v>589</v>
       </c>
-      <c r="B187" s="11" t="s">
-        <v>590</v>
-      </c>
       <c r="C187" s="5" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="E187" t="str">
         <f t="shared" si="6"/>
@@ -6335,10 +6335,10 @@
     </row>
     <row r="190" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A190" s="5" t="s">
+        <v>612</v>
+      </c>
+      <c r="B190" s="5" t="s">
         <v>613</v>
-      </c>
-      <c r="B190" s="5" t="s">
-        <v>614</v>
       </c>
       <c r="C190" s="5" t="s">
         <v>292</v>
@@ -6451,13 +6451,13 @@
         <v>280</v>
       </c>
       <c r="B197" s="5" t="s">
+        <v>849</v>
+      </c>
+      <c r="C197" s="5" t="s">
+        <v>422</v>
+      </c>
+      <c r="D197" s="17" t="s">
         <v>850</v>
-      </c>
-      <c r="C197" s="5" t="s">
-        <v>423</v>
-      </c>
-      <c r="D197" s="17" t="s">
-        <v>851</v>
       </c>
       <c r="E197">
         <f t="shared" si="6"/>
@@ -6466,13 +6466,13 @@
     </row>
     <row r="198" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A198" s="11" t="s">
+        <v>561</v>
+      </c>
+      <c r="B198" s="11" t="s">
         <v>562</v>
       </c>
-      <c r="B198" s="11" t="s">
-        <v>563</v>
-      </c>
       <c r="C198" s="5" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="E198" t="str">
         <f t="shared" si="6"/>
@@ -6481,10 +6481,10 @@
     </row>
     <row r="199" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A199" s="5" t="s">
+        <v>454</v>
+      </c>
+      <c r="B199" s="5" t="s">
         <v>455</v>
-      </c>
-      <c r="B199" s="5" t="s">
-        <v>456</v>
       </c>
       <c r="C199" s="5" t="s">
         <v>182</v>
@@ -6496,13 +6496,13 @@
     </row>
     <row r="200" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A200" s="5" t="s">
+        <v>690</v>
+      </c>
+      <c r="B200" s="5" t="s">
         <v>691</v>
       </c>
-      <c r="B200" s="5" t="s">
+      <c r="C200" s="5" t="s">
         <v>692</v>
-      </c>
-      <c r="C200" s="5" t="s">
-        <v>693</v>
       </c>
       <c r="E200" t="str">
         <f t="shared" si="6"/>
@@ -6526,10 +6526,10 @@
     </row>
     <row r="202" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A202" s="5" t="s">
+        <v>643</v>
+      </c>
+      <c r="B202" s="5" t="s">
         <v>644</v>
-      </c>
-      <c r="B202" s="5" t="s">
-        <v>645</v>
       </c>
       <c r="C202" s="5" t="s">
         <v>292</v>
@@ -6571,10 +6571,10 @@
     </row>
     <row r="205" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A205" s="5" t="s">
+        <v>780</v>
+      </c>
+      <c r="B205" s="5" t="s">
         <v>781</v>
-      </c>
-      <c r="B205" s="5" t="s">
-        <v>782</v>
       </c>
       <c r="C205" s="5" t="s">
         <v>292</v>
@@ -6586,10 +6586,10 @@
     </row>
     <row r="206" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A206" s="5" t="s">
+        <v>456</v>
+      </c>
+      <c r="B206" s="5" t="s">
         <v>457</v>
-      </c>
-      <c r="B206" s="5" t="s">
-        <v>458</v>
       </c>
       <c r="C206" s="5" t="s">
         <v>182</v>
@@ -6601,10 +6601,10 @@
     </row>
     <row r="207" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A207" s="5" t="s">
+        <v>527</v>
+      </c>
+      <c r="B207" s="5" t="s">
         <v>528</v>
-      </c>
-      <c r="B207" s="5" t="s">
-        <v>529</v>
       </c>
       <c r="C207" s="5" t="s">
         <v>292</v>
@@ -6648,10 +6648,10 @@
     </row>
     <row r="210" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A210" s="5" t="s">
+        <v>782</v>
+      </c>
+      <c r="B210" s="5" t="s">
         <v>783</v>
-      </c>
-      <c r="B210" s="5" t="s">
-        <v>784</v>
       </c>
       <c r="C210" s="5" t="s">
         <v>292</v>
@@ -6663,10 +6663,10 @@
     </row>
     <row r="211" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A211" s="5" t="s">
+        <v>645</v>
+      </c>
+      <c r="B211" s="5" t="s">
         <v>646</v>
-      </c>
-      <c r="B211" s="5" t="s">
-        <v>647</v>
       </c>
       <c r="C211" s="5" t="s">
         <v>300</v>
@@ -6678,10 +6678,10 @@
     </row>
     <row r="212" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A212" s="5" t="s">
+        <v>629</v>
+      </c>
+      <c r="B212" s="5" t="s">
         <v>630</v>
-      </c>
-      <c r="B212" s="5" t="s">
-        <v>631</v>
       </c>
       <c r="C212" s="5" t="s">
         <v>292</v>
@@ -6693,10 +6693,10 @@
     </row>
     <row r="213" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A213" s="5" t="s">
+        <v>622</v>
+      </c>
+      <c r="B213" s="5" t="s">
         <v>623</v>
-      </c>
-      <c r="B213" s="5" t="s">
-        <v>624</v>
       </c>
       <c r="C213" s="5" t="s">
         <v>182</v>
@@ -6708,13 +6708,13 @@
     </row>
     <row r="214" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A214" s="11" t="s">
+        <v>563</v>
+      </c>
+      <c r="B214" s="11" t="s">
         <v>564</v>
       </c>
-      <c r="B214" s="11" t="s">
-        <v>565</v>
-      </c>
       <c r="C214" s="5" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="E214" t="str">
         <f t="shared" si="7"/>
@@ -6760,7 +6760,7 @@
         <v>3</v>
       </c>
       <c r="B217" s="5" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="C217" s="5" t="s">
         <v>292</v>
@@ -6837,10 +6837,10 @@
     </row>
     <row r="222" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A222" s="5" t="s">
+        <v>501</v>
+      </c>
+      <c r="B222" s="5" t="s">
         <v>502</v>
-      </c>
-      <c r="B222" s="5" t="s">
-        <v>503</v>
       </c>
       <c r="C222" s="5" t="s">
         <v>300</v>
@@ -6852,10 +6852,10 @@
     </row>
     <row r="223" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A223" s="5" t="s">
+        <v>631</v>
+      </c>
+      <c r="B223" s="5" t="s">
         <v>632</v>
-      </c>
-      <c r="B223" s="5" t="s">
-        <v>633</v>
       </c>
       <c r="C223" s="5" t="s">
         <v>292</v>
@@ -6914,10 +6914,10 @@
     </row>
     <row r="227" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A227" s="5" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="B227" s="5" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
       <c r="C227" s="5" t="s">
         <v>300</v>
@@ -6960,10 +6960,10 @@
     </row>
     <row r="230" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A230" s="5" t="s">
+        <v>665</v>
+      </c>
+      <c r="B230" s="5" t="s">
         <v>666</v>
-      </c>
-      <c r="B230" s="5" t="s">
-        <v>667</v>
       </c>
       <c r="C230" s="5" t="s">
         <v>300</v>
@@ -7007,13 +7007,13 @@
     </row>
     <row r="233" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A233" s="11" t="s">
+        <v>571</v>
+      </c>
+      <c r="B233" s="11" t="s">
         <v>572</v>
       </c>
-      <c r="B233" s="11" t="s">
-        <v>573</v>
-      </c>
       <c r="C233" s="5" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="E233" t="str">
         <f t="shared" si="7"/>
@@ -7072,10 +7072,10 @@
     </row>
     <row r="237" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A237" s="5" t="s">
+        <v>799</v>
+      </c>
+      <c r="B237" s="5" t="s">
         <v>800</v>
-      </c>
-      <c r="B237" s="5" t="s">
-        <v>801</v>
       </c>
       <c r="C237" s="5" t="s">
         <v>300</v>
@@ -7087,13 +7087,13 @@
     </row>
     <row r="238" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A238" s="5" t="s">
+        <v>765</v>
+      </c>
+      <c r="B238" s="5" t="s">
         <v>766</v>
       </c>
-      <c r="B238" s="5" t="s">
-        <v>767</v>
-      </c>
       <c r="C238" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="E238" t="str">
         <f t="shared" si="7"/>
@@ -7133,13 +7133,13 @@
     </row>
     <row r="241" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A241" s="11" t="s">
+        <v>576</v>
+      </c>
+      <c r="B241" s="11" t="s">
         <v>577</v>
       </c>
-      <c r="B241" s="11" t="s">
-        <v>578</v>
-      </c>
       <c r="C241" s="5" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="E241" t="str">
         <f t="shared" si="7"/>
@@ -7148,10 +7148,10 @@
     </row>
     <row r="242" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A242" s="5" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="B242" s="5" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="C242" s="5" t="s">
         <v>292</v>
@@ -7163,10 +7163,10 @@
     </row>
     <row r="243" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A243" s="5" t="s">
+        <v>656</v>
+      </c>
+      <c r="B243" s="5" t="s">
         <v>657</v>
-      </c>
-      <c r="B243" s="5" t="s">
-        <v>658</v>
       </c>
       <c r="C243" s="5" t="s">
         <v>292</v>
@@ -7208,10 +7208,10 @@
     </row>
     <row r="246" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A246" s="5" t="s">
+        <v>667</v>
+      </c>
+      <c r="B246" s="5" t="s">
         <v>668</v>
-      </c>
-      <c r="B246" s="5" t="s">
-        <v>669</v>
       </c>
       <c r="C246" s="5" t="s">
         <v>300</v>
@@ -7223,10 +7223,10 @@
     </row>
     <row r="247" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A247" s="5" t="s">
+        <v>801</v>
+      </c>
+      <c r="B247" s="5" t="s">
         <v>802</v>
-      </c>
-      <c r="B247" s="5" t="s">
-        <v>803</v>
       </c>
       <c r="C247" s="5" t="s">
         <v>300</v>
@@ -7253,10 +7253,10 @@
     </row>
     <row r="249" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A249" s="5" t="s">
+        <v>813</v>
+      </c>
+      <c r="B249" s="5" t="s">
         <v>814</v>
-      </c>
-      <c r="B249" s="5" t="s">
-        <v>815</v>
       </c>
       <c r="C249" s="5" t="s">
         <v>300</v>
@@ -7268,13 +7268,13 @@
     </row>
     <row r="250" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A250" s="5" t="s">
+        <v>525</v>
+      </c>
+      <c r="B250" s="5" t="s">
         <v>526</v>
       </c>
-      <c r="B250" s="5" t="s">
-        <v>527</v>
-      </c>
       <c r="C250" s="5" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E250" t="str">
         <f t="shared" si="8"/>
@@ -7326,13 +7326,13 @@
     </row>
     <row r="254" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A254" s="5" t="s">
+        <v>809</v>
+      </c>
+      <c r="B254" s="5" t="s">
         <v>810</v>
       </c>
-      <c r="B254" s="5" t="s">
-        <v>811</v>
-      </c>
       <c r="C254" s="5" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E254" t="str">
         <f t="shared" ref="E254:E270" si="9">IF(AND(A254=A253,A254&lt;&gt;""),1,"")</f>
@@ -7341,10 +7341,10 @@
     </row>
     <row r="255" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A255" s="5" t="s">
+        <v>709</v>
+      </c>
+      <c r="B255" s="5" t="s">
         <v>710</v>
-      </c>
-      <c r="B255" s="5" t="s">
-        <v>711</v>
       </c>
       <c r="C255" s="5" t="s">
         <v>292</v>
@@ -7356,7 +7356,7 @@
     </row>
     <row r="256" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A256" s="5" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="B256" s="5" t="s">
         <v>299</v>
@@ -7371,10 +7371,10 @@
     </row>
     <row r="257" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A257" s="5" t="s">
+        <v>435</v>
+      </c>
+      <c r="B257" s="5" t="s">
         <v>436</v>
-      </c>
-      <c r="B257" s="5" t="s">
-        <v>437</v>
       </c>
       <c r="C257" s="5" t="s">
         <v>292</v>
@@ -7461,10 +7461,10 @@
     </row>
     <row r="263" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A263" s="5" t="s">
+        <v>679</v>
+      </c>
+      <c r="B263" s="5" t="s">
         <v>680</v>
-      </c>
-      <c r="B263" s="5" t="s">
-        <v>681</v>
       </c>
       <c r="C263" s="5" t="s">
         <v>292</v>
@@ -7476,13 +7476,13 @@
     </row>
     <row r="264" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A264" s="5" t="s">
+        <v>789</v>
+      </c>
+      <c r="B264" s="5" t="s">
         <v>790</v>
       </c>
-      <c r="B264" s="5" t="s">
-        <v>791</v>
-      </c>
       <c r="C264" s="5" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="E264" t="str">
         <f t="shared" si="9"/>
@@ -7521,10 +7521,10 @@
     </row>
     <row r="267" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A267" s="5" t="s">
+        <v>487</v>
+      </c>
+      <c r="B267" s="5" t="s">
         <v>488</v>
-      </c>
-      <c r="B267" s="5" t="s">
-        <v>489</v>
       </c>
       <c r="C267" s="5" t="s">
         <v>292</v>
@@ -7536,10 +7536,10 @@
     </row>
     <row r="268" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A268" s="5" t="s">
+        <v>652</v>
+      </c>
+      <c r="B268" s="5" t="s">
         <v>653</v>
-      </c>
-      <c r="B268" s="5" t="s">
-        <v>654</v>
       </c>
       <c r="C268" s="5" t="s">
         <v>292</v>
@@ -7567,10 +7567,10 @@
     </row>
     <row r="270" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A270" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="B270" s="5" t="s">
         <v>659</v>
-      </c>
-      <c r="B270" s="5" t="s">
-        <v>660</v>
       </c>
       <c r="C270" s="5" t="s">
         <v>292</v>
@@ -7582,7 +7582,7 @@
     </row>
     <row r="271" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A271" s="6" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="B271" s="5" t="s">
         <v>31</v>
@@ -7598,10 +7598,10 @@
     </row>
     <row r="272" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A272" s="11" t="s">
+        <v>593</v>
+      </c>
+      <c r="B272" s="12" t="s">
         <v>594</v>
-      </c>
-      <c r="B272" s="12" t="s">
-        <v>595</v>
       </c>
       <c r="C272" s="5" t="s">
         <v>292</v>
@@ -7628,10 +7628,10 @@
     </row>
     <row r="274" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A274" s="5" t="s">
+        <v>541</v>
+      </c>
+      <c r="B274" s="5" t="s">
         <v>542</v>
-      </c>
-      <c r="B274" s="5" t="s">
-        <v>543</v>
       </c>
       <c r="C274" s="5" t="s">
         <v>300</v>
@@ -7659,10 +7659,10 @@
     </row>
     <row r="276" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A276" s="5" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="B276" s="5" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="C276" s="5" t="s">
         <v>292</v>
@@ -7674,10 +7674,10 @@
     </row>
     <row r="277" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A277" s="5" t="s">
+        <v>654</v>
+      </c>
+      <c r="B277" s="5" t="s">
         <v>655</v>
-      </c>
-      <c r="B277" s="5" t="s">
-        <v>656</v>
       </c>
       <c r="C277" s="5" t="s">
         <v>292</v>
@@ -7689,10 +7689,10 @@
     </row>
     <row r="278" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A278" s="5" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="B278" s="5" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="C278" s="5" t="s">
         <v>292</v>
@@ -7704,10 +7704,10 @@
     </row>
     <row r="279" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A279" s="5" t="s">
+        <v>797</v>
+      </c>
+      <c r="B279" s="5" t="s">
         <v>798</v>
-      </c>
-      <c r="B279" s="5" t="s">
-        <v>799</v>
       </c>
       <c r="C279" s="5" t="s">
         <v>300</v>
@@ -7719,10 +7719,10 @@
     </row>
     <row r="280" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A280" s="5" t="s">
+        <v>739</v>
+      </c>
+      <c r="B280" s="5" t="s">
         <v>740</v>
-      </c>
-      <c r="B280" s="5" t="s">
-        <v>741</v>
       </c>
       <c r="C280" s="5" t="s">
         <v>300</v>
@@ -7734,10 +7734,10 @@
     </row>
     <row r="281" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A281" s="5" t="s">
+        <v>757</v>
+      </c>
+      <c r="B281" s="5" t="s">
         <v>758</v>
-      </c>
-      <c r="B281" s="5" t="s">
-        <v>759</v>
       </c>
       <c r="C281" s="5" t="s">
         <v>300</v>
@@ -7749,10 +7749,10 @@
     </row>
     <row r="282" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A282" s="5" t="s">
+        <v>828</v>
+      </c>
+      <c r="B282" s="5" t="s">
         <v>829</v>
-      </c>
-      <c r="B282" s="5" t="s">
-        <v>830</v>
       </c>
       <c r="C282" s="5" t="s">
         <v>300</v>
@@ -7780,10 +7780,10 @@
     </row>
     <row r="284" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A284" s="5" t="s">
+        <v>784</v>
+      </c>
+      <c r="B284" s="5" t="s">
         <v>785</v>
-      </c>
-      <c r="B284" s="5" t="s">
-        <v>786</v>
       </c>
       <c r="C284" s="5" t="s">
         <v>292</v>
@@ -7825,10 +7825,10 @@
     </row>
     <row r="287" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A287" s="5" t="s">
+        <v>605</v>
+      </c>
+      <c r="B287" s="5" t="s">
         <v>606</v>
-      </c>
-      <c r="B287" s="5" t="s">
-        <v>607</v>
       </c>
       <c r="C287" s="5" t="s">
         <v>292</v>
@@ -7840,13 +7840,13 @@
     </row>
     <row r="288" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A288" s="5" t="s">
+        <v>763</v>
+      </c>
+      <c r="B288" s="5" t="s">
         <v>764</v>
       </c>
-      <c r="B288" s="5" t="s">
-        <v>765</v>
-      </c>
       <c r="C288" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="E288" t="str">
         <f t="shared" si="10"/>
@@ -7855,10 +7855,10 @@
     </row>
     <row r="289" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A289" s="5" t="s">
+        <v>843</v>
+      </c>
+      <c r="B289" s="5" t="s">
         <v>844</v>
-      </c>
-      <c r="B289" s="5" t="s">
-        <v>845</v>
       </c>
       <c r="C289" s="5" t="s">
         <v>292</v>
@@ -7885,13 +7885,13 @@
     </row>
     <row r="291" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A291" s="11" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="B291" s="11" t="s">
         <v>378</v>
       </c>
       <c r="C291" s="5" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="E291">
         <f t="shared" si="10"/>
@@ -7900,10 +7900,10 @@
     </row>
     <row r="292" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A292" s="5" t="s">
+        <v>759</v>
+      </c>
+      <c r="B292" s="5" t="s">
         <v>760</v>
-      </c>
-      <c r="B292" s="5" t="s">
-        <v>761</v>
       </c>
       <c r="C292" s="5" t="s">
         <v>300</v>
@@ -7915,10 +7915,10 @@
     </row>
     <row r="293" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A293" s="5" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="B293" s="5" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
       <c r="C293" s="5" t="s">
         <v>300</v>
@@ -7945,10 +7945,10 @@
     </row>
     <row r="295" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A295" s="5" t="s">
+        <v>601</v>
+      </c>
+      <c r="B295" s="5" t="s">
         <v>602</v>
-      </c>
-      <c r="B295" s="5" t="s">
-        <v>603</v>
       </c>
       <c r="C295" s="5" t="s">
         <v>300</v>
@@ -7960,10 +7960,10 @@
     </row>
     <row r="296" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A296" s="5" t="s">
+        <v>443</v>
+      </c>
+      <c r="B296" s="5" t="s">
         <v>444</v>
-      </c>
-      <c r="B296" s="5" t="s">
-        <v>445</v>
       </c>
       <c r="C296" s="5" t="s">
         <v>300</v>
@@ -8005,16 +8005,16 @@
     </row>
     <row r="299" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A299" s="5" t="s">
+        <v>771</v>
+      </c>
+      <c r="B299" s="5" t="s">
         <v>772</v>
-      </c>
-      <c r="B299" s="5" t="s">
-        <v>773</v>
       </c>
       <c r="C299" s="5" t="s">
         <v>292</v>
       </c>
       <c r="D299" s="5" t="s">
-        <v>774</v>
+        <v>773</v>
       </c>
       <c r="E299" t="str">
         <f t="shared" si="10"/>
@@ -8023,10 +8023,10 @@
     </row>
     <row r="300" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A300" s="5" t="s">
+        <v>704</v>
+      </c>
+      <c r="B300" s="5" t="s">
         <v>705</v>
-      </c>
-      <c r="B300" s="5" t="s">
-        <v>706</v>
       </c>
       <c r="C300" s="5" t="s">
         <v>300</v>
@@ -8038,13 +8038,13 @@
     </row>
     <row r="301" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A301" s="11" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="B301" s="11" t="s">
         <v>172</v>
       </c>
       <c r="C301" s="5" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="E301" t="str">
         <f t="shared" si="10"/>
@@ -8053,13 +8053,13 @@
     </row>
     <row r="302" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A302" s="5" t="s">
+        <v>669</v>
+      </c>
+      <c r="B302" s="5" t="s">
         <v>670</v>
       </c>
-      <c r="B302" s="5" t="s">
-        <v>671</v>
-      </c>
       <c r="C302" s="5" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E302" t="str">
         <f t="shared" si="10"/>
@@ -8068,10 +8068,10 @@
     </row>
     <row r="303" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A303" s="5" t="s">
+        <v>839</v>
+      </c>
+      <c r="B303" s="5" t="s">
         <v>840</v>
-      </c>
-      <c r="B303" s="5" t="s">
-        <v>841</v>
       </c>
       <c r="C303" s="5" t="s">
         <v>292</v>
@@ -8083,10 +8083,10 @@
     </row>
     <row r="304" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A304" s="5" t="s">
+        <v>715</v>
+      </c>
+      <c r="B304" s="5" t="s">
         <v>716</v>
-      </c>
-      <c r="B304" s="5" t="s">
-        <v>717</v>
       </c>
       <c r="C304" s="5" t="s">
         <v>300</v>
@@ -8113,10 +8113,10 @@
     </row>
     <row r="306" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A306" s="5" t="s">
+        <v>499</v>
+      </c>
+      <c r="B306" s="5" t="s">
         <v>500</v>
-      </c>
-      <c r="B306" s="5" t="s">
-        <v>501</v>
       </c>
       <c r="C306" s="5" t="s">
         <v>292</v>
@@ -8159,13 +8159,13 @@
     </row>
     <row r="309" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A309" s="5" t="s">
+        <v>424</v>
+      </c>
+      <c r="B309" s="5" t="s">
         <v>425</v>
       </c>
-      <c r="B309" s="5" t="s">
-        <v>426</v>
-      </c>
       <c r="C309" s="5" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E309">
         <f t="shared" si="10"/>
@@ -8183,7 +8183,7 @@
         <v>292</v>
       </c>
       <c r="D310" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="E310">
         <f t="shared" si="10"/>
@@ -8192,10 +8192,10 @@
     </row>
     <row r="311" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A311" s="5" t="s">
+        <v>543</v>
+      </c>
+      <c r="B311" s="5" t="s">
         <v>544</v>
-      </c>
-      <c r="B311" s="5" t="s">
-        <v>545</v>
       </c>
       <c r="C311" s="5" t="s">
         <v>292</v>
@@ -8238,10 +8238,10 @@
     </row>
     <row r="314" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A314" s="5" t="s">
+        <v>733</v>
+      </c>
+      <c r="B314" s="5" t="s">
         <v>734</v>
-      </c>
-      <c r="B314" s="5" t="s">
-        <v>735</v>
       </c>
       <c r="C314" s="5" t="s">
         <v>300</v>
@@ -8253,10 +8253,10 @@
     </row>
     <row r="315" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A315" s="5" t="s">
+        <v>731</v>
+      </c>
+      <c r="B315" s="5" t="s">
         <v>732</v>
-      </c>
-      <c r="B315" s="5" t="s">
-        <v>733</v>
       </c>
       <c r="C315" s="5" t="s">
         <v>292</v>
@@ -8299,13 +8299,13 @@
     </row>
     <row r="318" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A318" s="5" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="B318" s="5" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="C318" s="5" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="D318" s="5"/>
       <c r="E318" t="str">
@@ -8347,13 +8347,13 @@
     </row>
     <row r="321" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A321" s="5" t="s">
+        <v>847</v>
+      </c>
+      <c r="B321" s="5" t="s">
         <v>848</v>
       </c>
-      <c r="B321" s="5" t="s">
-        <v>849</v>
-      </c>
       <c r="C321" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="E321" t="str">
         <f t="shared" si="10"/>
@@ -8378,13 +8378,13 @@
     </row>
     <row r="323" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A323" s="11" t="s">
+        <v>554</v>
+      </c>
+      <c r="B323" s="11" t="s">
         <v>555</v>
       </c>
-      <c r="B323" s="11" t="s">
-        <v>556</v>
-      </c>
       <c r="C323" s="5" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="E323" t="str">
         <f t="shared" si="10"/>
@@ -8393,13 +8393,13 @@
     </row>
     <row r="324" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A324" s="11" t="s">
+        <v>586</v>
+      </c>
+      <c r="B324" s="11" t="s">
         <v>587</v>
       </c>
-      <c r="B324" s="11" t="s">
-        <v>588</v>
-      </c>
       <c r="C324" s="5" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="E324" t="str">
         <f t="shared" si="10"/>
@@ -8408,10 +8408,10 @@
     </row>
     <row r="325" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A325" s="5" t="s">
+        <v>517</v>
+      </c>
+      <c r="B325" s="5" t="s">
         <v>518</v>
-      </c>
-      <c r="B325" s="5" t="s">
-        <v>519</v>
       </c>
       <c r="C325" s="5" t="s">
         <v>292</v>
@@ -8423,10 +8423,10 @@
     </row>
     <row r="326" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A326" s="5" t="s">
+        <v>807</v>
+      </c>
+      <c r="B326" s="5" t="s">
         <v>808</v>
-      </c>
-      <c r="B326" s="5" t="s">
-        <v>809</v>
       </c>
       <c r="C326" s="5" t="s">
         <v>300</v>
@@ -8453,10 +8453,10 @@
     </row>
     <row r="328" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A328" s="5" t="s">
+        <v>824</v>
+      </c>
+      <c r="B328" s="5" t="s">
         <v>825</v>
-      </c>
-      <c r="B328" s="5" t="s">
-        <v>826</v>
       </c>
       <c r="C328" s="5" t="s">
         <v>292</v>
@@ -8468,10 +8468,10 @@
     </row>
     <row r="329" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A329" s="5" t="s">
+        <v>723</v>
+      </c>
+      <c r="B329" s="5" t="s">
         <v>724</v>
-      </c>
-      <c r="B329" s="5" t="s">
-        <v>725</v>
       </c>
       <c r="C329" s="5" t="s">
         <v>300</v>
@@ -8499,10 +8499,10 @@
     </row>
     <row r="331" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A331" s="5" t="s">
+        <v>505</v>
+      </c>
+      <c r="B331" s="5" t="s">
         <v>506</v>
-      </c>
-      <c r="B331" s="5" t="s">
-        <v>507</v>
       </c>
       <c r="C331" s="5" t="s">
         <v>292</v>
@@ -8514,10 +8514,10 @@
     </row>
     <row r="332" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A332" s="5" t="s">
+        <v>531</v>
+      </c>
+      <c r="B332" s="5" t="s">
         <v>532</v>
-      </c>
-      <c r="B332" s="5" t="s">
-        <v>533</v>
       </c>
       <c r="C332" s="5" t="s">
         <v>292</v>
@@ -8560,10 +8560,10 @@
     </row>
     <row r="335" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A335" s="5" t="s">
+        <v>509</v>
+      </c>
+      <c r="B335" s="5" t="s">
         <v>510</v>
-      </c>
-      <c r="B335" s="5" t="s">
-        <v>511</v>
       </c>
       <c r="C335" s="5" t="s">
         <v>292</v>
@@ -8575,10 +8575,10 @@
     </row>
     <row r="336" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A336" s="5" t="s">
+        <v>511</v>
+      </c>
+      <c r="B336" s="5" t="s">
         <v>512</v>
-      </c>
-      <c r="B336" s="5" t="s">
-        <v>513</v>
       </c>
       <c r="C336" s="5" t="s">
         <v>292</v>
@@ -8590,13 +8590,13 @@
     </row>
     <row r="337" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A337" s="5" t="s">
+        <v>721</v>
+      </c>
+      <c r="B337" s="5" t="s">
         <v>722</v>
       </c>
-      <c r="B337" s="5" t="s">
-        <v>723</v>
-      </c>
       <c r="C337" s="5" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E337" t="str">
         <f t="shared" si="11"/>
@@ -8621,13 +8621,13 @@
     </row>
     <row r="339" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A339" s="11" t="s">
+        <v>578</v>
+      </c>
+      <c r="B339" s="11" t="s">
         <v>579</v>
       </c>
-      <c r="B339" s="11" t="s">
-        <v>580</v>
-      </c>
       <c r="C339" s="5" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="E339" t="str">
         <f t="shared" si="11"/>
@@ -8667,10 +8667,10 @@
     </row>
     <row r="342" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A342" s="5" t="s">
+        <v>519</v>
+      </c>
+      <c r="B342" s="5" t="s">
         <v>520</v>
-      </c>
-      <c r="B342" s="5" t="s">
-        <v>521</v>
       </c>
       <c r="C342" s="5" t="s">
         <v>292</v>
@@ -8682,10 +8682,10 @@
     </row>
     <row r="343" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A343" s="5" t="s">
+        <v>663</v>
+      </c>
+      <c r="B343" s="5" t="s">
         <v>664</v>
-      </c>
-      <c r="B343" s="5" t="s">
-        <v>665</v>
       </c>
       <c r="C343" s="5" t="s">
         <v>292</v>
@@ -8697,10 +8697,10 @@
     </row>
     <row r="344" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A344" s="5" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="B344" s="5" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="C344" s="5" t="s">
         <v>292</v>
@@ -8712,10 +8712,10 @@
     </row>
     <row r="345" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A345" s="5" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="B345" s="5" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C345" s="5" t="s">
         <v>292</v>
@@ -8727,10 +8727,10 @@
     </row>
     <row r="346" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A346" s="5" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="B346" s="5" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="C346" s="5" t="s">
         <v>292</v>
@@ -8758,10 +8758,10 @@
     </row>
     <row r="348" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A348" s="5" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="B348" s="5" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="C348" s="5" t="s">
         <v>300</v>
@@ -8773,10 +8773,10 @@
     </row>
     <row r="349" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A349" s="5" t="s">
+        <v>445</v>
+      </c>
+      <c r="B349" s="5" t="s">
         <v>446</v>
-      </c>
-      <c r="B349" s="5" t="s">
-        <v>447</v>
       </c>
       <c r="C349" s="5" t="s">
         <v>300</v>
@@ -8819,10 +8819,10 @@
     </row>
     <row r="352" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A352" s="5" t="s">
+        <v>493</v>
+      </c>
+      <c r="B352" s="5" t="s">
         <v>494</v>
-      </c>
-      <c r="B352" s="5" t="s">
-        <v>495</v>
       </c>
       <c r="C352" s="5" t="s">
         <v>292</v>
@@ -8850,13 +8850,13 @@
     </row>
     <row r="354" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A354" s="11" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="B354" s="11" t="s">
         <v>62</v>
       </c>
       <c r="C354" s="5" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="E354">
         <f t="shared" si="11"/>
@@ -9054,13 +9054,13 @@
     </row>
     <row r="367" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A367" s="5" t="s">
+        <v>426</v>
+      </c>
+      <c r="B367" s="5" t="s">
         <v>427</v>
       </c>
-      <c r="B367" s="5" t="s">
-        <v>428</v>
-      </c>
       <c r="C367" s="5" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E367">
         <f t="shared" si="11"/>
@@ -9069,13 +9069,13 @@
     </row>
     <row r="368" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A368" s="11" t="s">
+        <v>580</v>
+      </c>
+      <c r="B368" s="11" t="s">
         <v>581</v>
       </c>
-      <c r="B368" s="11" t="s">
-        <v>582</v>
-      </c>
       <c r="C368" s="5" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="E368" t="str">
         <f t="shared" si="11"/>
@@ -9099,10 +9099,10 @@
     </row>
     <row r="370" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A370" s="5" t="s">
+        <v>753</v>
+      </c>
+      <c r="B370" s="5" t="s">
         <v>754</v>
-      </c>
-      <c r="B370" s="5" t="s">
-        <v>755</v>
       </c>
       <c r="C370" s="5" t="s">
         <v>300</v>
@@ -9114,10 +9114,10 @@
     </row>
     <row r="371" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A371" s="5" t="s">
+        <v>698</v>
+      </c>
+      <c r="B371" s="5" t="s">
         <v>699</v>
-      </c>
-      <c r="B371" s="5" t="s">
-        <v>700</v>
       </c>
       <c r="C371" s="5" t="s">
         <v>300</v>
@@ -9145,10 +9145,10 @@
     </row>
     <row r="373" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A373" s="5" t="s">
+        <v>676</v>
+      </c>
+      <c r="B373" s="5" t="s">
         <v>677</v>
-      </c>
-      <c r="B373" s="5" t="s">
-        <v>678</v>
       </c>
       <c r="C373" s="5" t="s">
         <v>292</v>
@@ -9175,10 +9175,10 @@
     </row>
     <row r="375" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A375" s="5" t="s">
+        <v>624</v>
+      </c>
+      <c r="B375" s="5" t="s">
         <v>625</v>
-      </c>
-      <c r="B375" s="5" t="s">
-        <v>626</v>
       </c>
       <c r="C375" s="5" t="s">
         <v>292</v>
@@ -9221,10 +9221,10 @@
     </row>
     <row r="378" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A378" s="5" t="s">
+        <v>535</v>
+      </c>
+      <c r="B378" s="5" t="s">
         <v>536</v>
-      </c>
-      <c r="B378" s="5" t="s">
-        <v>537</v>
       </c>
       <c r="C378" s="5" t="s">
         <v>292</v>
@@ -9236,10 +9236,10 @@
     </row>
     <row r="379" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A379" s="5" t="s">
+        <v>514</v>
+      </c>
+      <c r="B379" s="5" t="s">
         <v>515</v>
-      </c>
-      <c r="B379" s="5" t="s">
-        <v>516</v>
       </c>
       <c r="C379" s="5" t="s">
         <v>156</v>
@@ -9251,10 +9251,10 @@
     </row>
     <row r="380" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A380" s="5" t="s">
+        <v>447</v>
+      </c>
+      <c r="B380" s="5" t="s">
         <v>448</v>
-      </c>
-      <c r="B380" s="5" t="s">
-        <v>449</v>
       </c>
       <c r="C380" s="5" t="s">
         <v>300</v>
@@ -9266,10 +9266,10 @@
     </row>
     <row r="381" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A381" s="5" t="s">
+        <v>719</v>
+      </c>
+      <c r="B381" s="5" t="s">
         <v>720</v>
-      </c>
-      <c r="B381" s="5" t="s">
-        <v>721</v>
       </c>
       <c r="C381" s="5" t="s">
         <v>292</v>
@@ -9281,10 +9281,10 @@
     </row>
     <row r="382" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A382" s="5" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="B382" s="5" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="C382" s="5" t="s">
         <v>300</v>
@@ -9296,10 +9296,10 @@
     </row>
     <row r="383" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A383" s="5" t="s">
+        <v>695</v>
+      </c>
+      <c r="B383" s="5" t="s">
         <v>696</v>
-      </c>
-      <c r="B383" s="5" t="s">
-        <v>697</v>
       </c>
       <c r="C383" s="5" t="s">
         <v>300</v>
@@ -9327,10 +9327,10 @@
     </row>
     <row r="385" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A385" s="5" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="B385" s="5" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="C385" s="5" t="s">
         <v>292</v>
@@ -9342,10 +9342,10 @@
     </row>
     <row r="386" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A386" s="5" t="s">
+        <v>727</v>
+      </c>
+      <c r="B386" s="5" t="s">
         <v>728</v>
-      </c>
-      <c r="B386" s="5" t="s">
-        <v>729</v>
       </c>
       <c r="C386" s="5" t="s">
         <v>292</v>
@@ -9373,13 +9373,13 @@
     </row>
     <row r="388" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A388" s="11" t="s">
+        <v>557</v>
+      </c>
+      <c r="B388" s="11" t="s">
         <v>558</v>
       </c>
-      <c r="B388" s="11" t="s">
-        <v>559</v>
-      </c>
       <c r="C388" s="5" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="E388" t="str">
         <f t="shared" si="11"/>
@@ -9388,13 +9388,13 @@
     </row>
     <row r="389" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A389" s="11" t="s">
+        <v>590</v>
+      </c>
+      <c r="B389" s="11" t="s">
         <v>591</v>
       </c>
-      <c r="B389" s="11" t="s">
+      <c r="C389" s="5" t="s">
         <v>592</v>
-      </c>
-      <c r="C389" s="5" t="s">
-        <v>593</v>
       </c>
       <c r="E389" t="str">
         <f t="shared" si="11"/>
@@ -9403,10 +9403,10 @@
     </row>
     <row r="390" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A390" s="5" t="s">
+        <v>650</v>
+      </c>
+      <c r="B390" s="5" t="s">
         <v>651</v>
-      </c>
-      <c r="B390" s="5" t="s">
-        <v>652</v>
       </c>
       <c r="C390" s="5" t="s">
         <v>292</v>
@@ -9433,10 +9433,10 @@
     </row>
     <row r="392" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A392" s="5" t="s">
+        <v>641</v>
+      </c>
+      <c r="B392" s="5" t="s">
         <v>642</v>
-      </c>
-      <c r="B392" s="5" t="s">
-        <v>643</v>
       </c>
       <c r="C392" s="5" t="s">
         <v>292</v>
@@ -9448,10 +9448,10 @@
     </row>
     <row r="393" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A393" s="5" t="s">
+        <v>603</v>
+      </c>
+      <c r="B393" s="5" t="s">
         <v>604</v>
-      </c>
-      <c r="B393" s="5" t="s">
-        <v>605</v>
       </c>
       <c r="C393" s="5" t="s">
         <v>292</v>
@@ -9463,10 +9463,10 @@
     </row>
     <row r="394" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A394" s="5" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
       <c r="B394" s="5" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="C394" s="5" t="s">
         <v>292</v>
@@ -9494,13 +9494,13 @@
     </row>
     <row r="396" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A396" s="5" t="s">
+        <v>761</v>
+      </c>
+      <c r="B396" s="5" t="s">
         <v>762</v>
       </c>
-      <c r="B396" s="5" t="s">
-        <v>763</v>
-      </c>
       <c r="C396" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="E396" t="str">
         <f t="shared" si="11"/>
@@ -9527,10 +9527,10 @@
     </row>
     <row r="398" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A398" s="5" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="B398" s="5" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="C398" s="5" t="s">
         <v>292</v>
@@ -9542,10 +9542,10 @@
     </row>
     <row r="399" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A399" s="5" t="s">
+        <v>791</v>
+      </c>
+      <c r="B399" t="s">
         <v>792</v>
-      </c>
-      <c r="B399" t="s">
-        <v>793</v>
       </c>
       <c r="C399" s="5" t="s">
         <v>300</v>
@@ -9557,10 +9557,10 @@
     </row>
     <row r="400" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A400" s="5" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="B400" s="5" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="C400" s="5" t="s">
         <v>292</v>
@@ -9618,13 +9618,13 @@
     </row>
     <row r="404" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A404" s="11" t="s">
+        <v>547</v>
+      </c>
+      <c r="B404" s="11" t="s">
         <v>548</v>
       </c>
-      <c r="B404" s="11" t="s">
-        <v>549</v>
-      </c>
       <c r="C404" s="5" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="E404" t="str">
         <f t="shared" si="12"/>
@@ -9648,10 +9648,10 @@
     </row>
     <row r="406" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A406" s="5" t="s">
+        <v>507</v>
+      </c>
+      <c r="B406" s="5" t="s">
         <v>508</v>
-      </c>
-      <c r="B406" s="5" t="s">
-        <v>509</v>
       </c>
       <c r="C406" s="5" t="s">
         <v>292</v>
@@ -9714,7 +9714,7 @@
         <v>32</v>
       </c>
       <c r="B410" s="5" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="C410" s="5" t="s">
         <v>290</v>
@@ -9726,7 +9726,7 @@
     </row>
     <row r="411" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A411" s="6" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="B411" s="5" t="s">
         <v>33</v>
@@ -9775,13 +9775,13 @@
     </row>
     <row r="414" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A414" s="5" t="s">
+        <v>735</v>
+      </c>
+      <c r="B414" s="5" t="s">
         <v>736</v>
       </c>
-      <c r="B414" s="5" t="s">
-        <v>737</v>
-      </c>
       <c r="C414" s="5" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E414" t="str">
         <f t="shared" si="12"/>
@@ -15665,7 +15665,7 @@
   <sheetData>
     <row r="1" spans="1:1" ht="60" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="15" x14ac:dyDescent="0.25">
@@ -15673,7 +15673,7 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
     </row>
     <row r="4" spans="1:1" ht="15" x14ac:dyDescent="0.25">
@@ -15683,22 +15683,22 @@
     </row>
     <row r="5" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" s="14" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" s="14" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" s="14" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.3">
@@ -15708,17 +15708,17 @@
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A13" s="14" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A14" s="14" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" s="15" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
wb fixes + INI end date-change
I realised that the end date is not inclussive so the Sims were missing 31/12 from the last year. I fixed it so that the child Sims don't inherent the same falacy.
</commit_message>
<xml_diff>
--- a/Mng/Acronyms.xlsx
+++ b/Mng/Acronyms.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Mng\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C912A69D-99BE-47FE-9E96-271DF7B7A24D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04DA40D1-B631-404E-BDE5-29FFB0A2531E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -307,7 +307,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4294947668" uniqueCount="856">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1878" uniqueCount="860">
   <si>
     <t>GW</t>
   </si>
@@ -2877,6 +2877,18 @@
   </si>
   <si>
     <t>l_</t>
+  </si>
+  <si>
+    <t>Su</t>
+  </si>
+  <si>
+    <t>Summer</t>
+  </si>
+  <si>
+    <t>Wi</t>
+  </si>
+  <si>
+    <t>Winter</t>
   </si>
 </sst>
 </file>
@@ -9893,9 +9905,14 @@
       </c>
     </row>
     <row r="421" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B421" s="5"/>
+      <c r="A421" s="5" t="s">
+        <v>856</v>
+      </c>
+      <c r="B421" s="5" t="s">
+        <v>857</v>
+      </c>
       <c r="C421" s="5" t="s">
-        <v>156</v>
+        <v>300</v>
       </c>
       <c r="E421" t="str">
         <f t="shared" si="12"/>
@@ -9903,9 +9920,14 @@
       </c>
     </row>
     <row r="422" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B422" s="5"/>
+      <c r="A422" s="5" t="s">
+        <v>858</v>
+      </c>
+      <c r="B422" s="5" t="s">
+        <v>859</v>
+      </c>
       <c r="C422" s="5" t="s">
-        <v>156</v>
+        <v>300</v>
       </c>
       <c r="E422" t="str">
         <f t="shared" si="12"/>

</xml_diff>